<commit_message>
Ajoute la famille asclépiade comestible, absente de l'audit initial
Huit occasions vérifiées, dont Gourmet Sauvage, qui transforme la même
plante par ses parties comestibles. Symbiose Herboristerie porte déjà deux
liens vers lasclay.com, dont un vers la page pilier, ce que l'audit
initial ignorait.

Le chiffrier passe de 72 à 80 occasions, rangs recalculés.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HLLDqBHKdaQwB3EuS9DRgG
</commit_message>
<xml_diff>
--- a/seo/backlinks-lasclay-audit.xlsx
+++ b/seo/backlinks-lasclay-audit.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Pistes à vérifier" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Opportunités'!$A$4:$U$76</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Opportunités'!$A$4:$U$84</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Pistes à vérifier'!$A$4:$H$32</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -23,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="18">
+  <fonts count="19">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -144,8 +144,14 @@
       <color rgb="00666666"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="000563C1"/>
+      <sz val="10"/>
+      <u val="single"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -191,8 +197,23 @@
         <fgColor rgb="00F4CCCC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9EAD3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -215,6 +236,20 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D9D9D9"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1">
@@ -226,7 +261,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="60">
+  <cellXfs count="70">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -404,6 +439,36 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -1438,7 +1503,7 @@
     </row>
     <row r="11" ht="61.5" customHeight="1" s="29">
       <c r="A11" s="33" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B11" s="34">
         <f>SUM(N11:Q11)</f>
@@ -1534,7 +1599,7 @@
     </row>
     <row r="12" ht="61.5" customHeight="1" s="29">
       <c r="A12" s="33" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B12" s="34">
         <f>SUM(N12:Q12)</f>
@@ -1630,7 +1695,7 @@
     </row>
     <row r="13" ht="61.5" customHeight="1" s="29">
       <c r="A13" s="33" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B13" s="34">
         <f>SUM(N13:Q13)</f>
@@ -1726,7 +1791,7 @@
     </row>
     <row r="14" ht="61.5" customHeight="1" s="29">
       <c r="A14" s="33" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B14" s="34">
         <f>SUM(N14:Q14)</f>
@@ -1818,7 +1883,7 @@
     </row>
     <row r="15" ht="61.5" customHeight="1" s="29">
       <c r="A15" s="33" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B15" s="34">
         <f>SUM(N15:Q15)</f>
@@ -1914,7 +1979,7 @@
     </row>
     <row r="16" ht="61.5" customHeight="1" s="29">
       <c r="A16" s="33" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B16" s="34">
         <f>SUM(N16:Q16)</f>
@@ -2010,7 +2075,7 @@
     </row>
     <row r="17" ht="61.5" customHeight="1" s="29">
       <c r="A17" s="33" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B17" s="34">
         <f>SUM(N17:Q17)</f>
@@ -2106,7 +2171,7 @@
     </row>
     <row r="18" ht="61.5" customHeight="1" s="29">
       <c r="A18" s="33" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B18" s="34">
         <f>SUM(N18:Q18)</f>
@@ -2198,7 +2263,7 @@
     </row>
     <row r="19" ht="61.5" customHeight="1" s="29">
       <c r="A19" s="33" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B19" s="34">
         <f>SUM(N19:Q19)</f>
@@ -2294,7 +2359,7 @@
     </row>
     <row r="20" ht="61.5" customHeight="1" s="29">
       <c r="A20" s="33" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B20" s="34">
         <f>SUM(N20:Q20)</f>
@@ -2390,7 +2455,7 @@
     </row>
     <row r="21" ht="61.5" customHeight="1" s="29">
       <c r="A21" s="33" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B21" s="34">
         <f>SUM(N21:Q21)</f>
@@ -2486,7 +2551,7 @@
     </row>
     <row r="22" ht="61.5" customHeight="1" s="29">
       <c r="A22" s="33" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B22" s="34">
         <f>SUM(N22:Q22)</f>
@@ -2582,7 +2647,7 @@
     </row>
     <row r="23" ht="61.5" customHeight="1" s="29">
       <c r="A23" s="33" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B23" s="34">
         <f>SUM(N23:Q23)</f>
@@ -2678,7 +2743,7 @@
     </row>
     <row r="24" ht="61.5" customHeight="1" s="29">
       <c r="A24" s="33" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B24" s="34">
         <f>SUM(N24:Q24)</f>
@@ -2774,7 +2839,7 @@
     </row>
     <row r="25" ht="61.5" customHeight="1" s="29">
       <c r="A25" s="33" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B25" s="34">
         <f>SUM(N25:Q25)</f>
@@ -2870,7 +2935,7 @@
     </row>
     <row r="26" ht="61.5" customHeight="1" s="29">
       <c r="A26" s="43" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B26" s="44">
         <f>SUM(N26:Q26)</f>
@@ -2966,7 +3031,7 @@
     </row>
     <row r="27" ht="61.5" customHeight="1" s="29">
       <c r="A27" s="43" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B27" s="44">
         <f>SUM(N27:Q27)</f>
@@ -3062,7 +3127,7 @@
     </row>
     <row r="28" ht="61.5" customHeight="1" s="29">
       <c r="A28" s="43" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B28" s="44">
         <f>SUM(N28:Q28)</f>
@@ -3154,7 +3219,7 @@
     </row>
     <row r="29" ht="61.5" customHeight="1" s="29">
       <c r="A29" s="43" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B29" s="44">
         <f>SUM(N29:Q29)</f>
@@ -3246,7 +3311,7 @@
     </row>
     <row r="30" ht="61.5" customHeight="1" s="29">
       <c r="A30" s="43" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B30" s="44">
         <f>SUM(N30:Q30)</f>
@@ -3342,7 +3407,7 @@
     </row>
     <row r="31" ht="61.5" customHeight="1" s="29">
       <c r="A31" s="43" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B31" s="44">
         <f>SUM(N31:Q31)</f>
@@ -3438,7 +3503,7 @@
     </row>
     <row r="32" ht="61.5" customHeight="1" s="29">
       <c r="A32" s="43" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="B32" s="44">
         <f>SUM(N32:Q32)</f>
@@ -3530,7 +3595,7 @@
     </row>
     <row r="33" ht="61.5" customHeight="1" s="29">
       <c r="A33" s="43" t="n">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="B33" s="44">
         <f>SUM(N33:Q33)</f>
@@ -3626,7 +3691,7 @@
     </row>
     <row r="34" ht="61.5" customHeight="1" s="29">
       <c r="A34" s="43" t="n">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="B34" s="44">
         <f>SUM(N34:Q34)</f>
@@ -3722,7 +3787,7 @@
     </row>
     <row r="35" ht="61.5" customHeight="1" s="29">
       <c r="A35" s="43" t="n">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B35" s="44">
         <f>SUM(N35:Q35)</f>
@@ -3818,7 +3883,7 @@
     </row>
     <row r="36" ht="61.5" customHeight="1" s="29">
       <c r="A36" s="43" t="n">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B36" s="44">
         <f>SUM(N36:Q36)</f>
@@ -3910,7 +3975,7 @@
     </row>
     <row r="37" ht="61.5" customHeight="1" s="29">
       <c r="A37" s="43" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="B37" s="44">
         <f>SUM(N37:Q37)</f>
@@ -4006,7 +4071,7 @@
     </row>
     <row r="38" ht="61.5" customHeight="1" s="29">
       <c r="A38" s="43" t="n">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="B38" s="44">
         <f>SUM(N38:Q38)</f>
@@ -4102,7 +4167,7 @@
     </row>
     <row r="39" ht="61.5" customHeight="1" s="29">
       <c r="A39" s="43" t="n">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="B39" s="44">
         <f>SUM(N39:Q39)</f>
@@ -4198,7 +4263,7 @@
     </row>
     <row r="40" ht="61.5" customHeight="1" s="29">
       <c r="A40" s="43" t="n">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="B40" s="44">
         <f>SUM(N40:Q40)</f>
@@ -4294,7 +4359,7 @@
     </row>
     <row r="41" ht="61.5" customHeight="1" s="29">
       <c r="A41" s="43" t="n">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="B41" s="44">
         <f>SUM(N41:Q41)</f>
@@ -4390,7 +4455,7 @@
     </row>
     <row r="42" ht="61.5" customHeight="1" s="29">
       <c r="A42" s="43" t="n">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="B42" s="44">
         <f>SUM(N42:Q42)</f>
@@ -4486,7 +4551,7 @@
     </row>
     <row r="43" ht="61.5" customHeight="1" s="29">
       <c r="A43" s="43" t="n">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="B43" s="44">
         <f>SUM(N43:Q43)</f>
@@ -4582,7 +4647,7 @@
     </row>
     <row r="44" ht="61.5" customHeight="1" s="29">
       <c r="A44" s="43" t="n">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="B44" s="44">
         <f>SUM(N44:Q44)</f>
@@ -4678,7 +4743,7 @@
     </row>
     <row r="45" ht="61.5" customHeight="1" s="29">
       <c r="A45" s="43" t="n">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="B45" s="44">
         <f>SUM(N45:Q45)</f>
@@ -4774,7 +4839,7 @@
     </row>
     <row r="46" ht="61.5" customHeight="1" s="29">
       <c r="A46" s="43" t="n">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="B46" s="44">
         <f>SUM(N46:Q46)</f>
@@ -4870,7 +4935,7 @@
     </row>
     <row r="47" ht="61.5" customHeight="1" s="29">
       <c r="A47" s="43" t="n">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="B47" s="44">
         <f>SUM(N47:Q47)</f>
@@ -4966,7 +5031,7 @@
     </row>
     <row r="48" ht="61.5" customHeight="1" s="29">
       <c r="A48" s="43" t="n">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="B48" s="44">
         <f>SUM(N48:Q48)</f>
@@ -5062,7 +5127,7 @@
     </row>
     <row r="49" ht="61.5" customHeight="1" s="29">
       <c r="A49" s="43" t="n">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="B49" s="44">
         <f>SUM(N49:Q49)</f>
@@ -5158,7 +5223,7 @@
     </row>
     <row r="50" ht="61.5" customHeight="1" s="29">
       <c r="A50" s="43" t="n">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="B50" s="44">
         <f>SUM(N50:Q50)</f>
@@ -5254,7 +5319,7 @@
     </row>
     <row r="51" ht="61.5" customHeight="1" s="29">
       <c r="A51" s="43" t="n">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="B51" s="44">
         <f>SUM(N51:Q51)</f>
@@ -5350,7 +5415,7 @@
     </row>
     <row r="52" ht="61.5" customHeight="1" s="29">
       <c r="A52" s="43" t="n">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="B52" s="44">
         <f>SUM(N52:Q52)</f>
@@ -5446,7 +5511,7 @@
     </row>
     <row r="53" ht="61.5" customHeight="1" s="29">
       <c r="A53" s="43" t="n">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="B53" s="44">
         <f>SUM(N53:Q53)</f>
@@ -5542,7 +5607,7 @@
     </row>
     <row r="54" ht="61.5" customHeight="1" s="29">
       <c r="A54" s="43" t="n">
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="B54" s="44">
         <f>SUM(N54:Q54)</f>
@@ -5638,7 +5703,7 @@
     </row>
     <row r="55" ht="61.5" customHeight="1" s="29">
       <c r="A55" s="43" t="n">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="B55" s="44">
         <f>SUM(N55:Q55)</f>
@@ -5734,7 +5799,7 @@
     </row>
     <row r="56" ht="61.5" customHeight="1" s="29">
       <c r="A56" s="43" t="n">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="B56" s="44">
         <f>SUM(N56:Q56)</f>
@@ -5830,7 +5895,7 @@
     </row>
     <row r="57" ht="61.5" customHeight="1" s="29">
       <c r="A57" s="43" t="n">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="B57" s="44">
         <f>SUM(N57:Q57)</f>
@@ -5926,7 +5991,7 @@
     </row>
     <row r="58" ht="61.5" customHeight="1" s="29">
       <c r="A58" s="43" t="n">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="B58" s="44">
         <f>SUM(N58:Q58)</f>
@@ -6022,7 +6087,7 @@
     </row>
     <row r="59" ht="61.5" customHeight="1" s="29">
       <c r="A59" s="43" t="n">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="B59" s="44">
         <f>SUM(N59:Q59)</f>
@@ -6118,7 +6183,7 @@
     </row>
     <row r="60" ht="61.5" customHeight="1" s="29">
       <c r="A60" s="43" t="n">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="B60" s="44">
         <f>SUM(N60:Q60)</f>
@@ -6214,7 +6279,7 @@
     </row>
     <row r="61" ht="61.5" customHeight="1" s="29">
       <c r="A61" s="43" t="n">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="B61" s="44">
         <f>SUM(N61:Q61)</f>
@@ -6310,7 +6375,7 @@
     </row>
     <row r="62" ht="61.5" customHeight="1" s="29">
       <c r="A62" s="43" t="n">
-        <v>58</v>
+        <v>65</v>
       </c>
       <c r="B62" s="44">
         <f>SUM(N62:Q62)</f>
@@ -6406,7 +6471,7 @@
     </row>
     <row r="63" ht="61.5" customHeight="1" s="29">
       <c r="A63" s="43" t="n">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="B63" s="44">
         <f>SUM(N63:Q63)</f>
@@ -6502,7 +6567,7 @@
     </row>
     <row r="64" ht="61.5" customHeight="1" s="29">
       <c r="A64" s="45" t="n">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="B64" s="46">
         <f>SUM(N64:Q64)</f>
@@ -6598,7 +6663,7 @@
     </row>
     <row r="65" ht="61.5" customHeight="1" s="29">
       <c r="A65" s="45" t="n">
-        <v>61</v>
+        <v>68</v>
       </c>
       <c r="B65" s="46">
         <f>SUM(N65:Q65)</f>
@@ -6694,7 +6759,7 @@
     </row>
     <row r="66" ht="61.5" customHeight="1" s="29">
       <c r="A66" s="45" t="n">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="B66" s="46">
         <f>SUM(N66:Q66)</f>
@@ -6790,7 +6855,7 @@
     </row>
     <row r="67" ht="61.5" customHeight="1" s="29">
       <c r="A67" s="45" t="n">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="B67" s="46">
         <f>SUM(N67:Q67)</f>
@@ -6886,7 +6951,7 @@
     </row>
     <row r="68" ht="61.5" customHeight="1" s="29">
       <c r="A68" s="45" t="n">
-        <v>64</v>
+        <v>71</v>
       </c>
       <c r="B68" s="46">
         <f>SUM(N68:Q68)</f>
@@ -6982,7 +7047,7 @@
     </row>
     <row r="69" ht="61.5" customHeight="1" s="29">
       <c r="A69" s="45" t="n">
-        <v>65</v>
+        <v>72</v>
       </c>
       <c r="B69" s="46">
         <f>SUM(N69:Q69)</f>
@@ -7078,7 +7143,7 @@
     </row>
     <row r="70" ht="61.5" customHeight="1" s="29">
       <c r="A70" s="45" t="n">
-        <v>66</v>
+        <v>74</v>
       </c>
       <c r="B70" s="46">
         <f>SUM(N70:Q70)</f>
@@ -7174,7 +7239,7 @@
     </row>
     <row r="71" ht="61.5" customHeight="1" s="29">
       <c r="A71" s="45" t="n">
-        <v>67</v>
+        <v>75</v>
       </c>
       <c r="B71" s="46">
         <f>SUM(N71:Q71)</f>
@@ -7270,7 +7335,7 @@
     </row>
     <row r="72" ht="61.5" customHeight="1" s="29">
       <c r="A72" s="45" t="n">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="B72" s="46">
         <f>SUM(N72:Q72)</f>
@@ -7366,7 +7431,7 @@
     </row>
     <row r="73" ht="61.5" customHeight="1" s="29">
       <c r="A73" s="45" t="n">
-        <v>69</v>
+        <v>77</v>
       </c>
       <c r="B73" s="46">
         <f>SUM(N73:Q73)</f>
@@ -7462,7 +7527,7 @@
     </row>
     <row r="74" ht="61.5" customHeight="1" s="29">
       <c r="A74" s="45" t="n">
-        <v>70</v>
+        <v>78</v>
       </c>
       <c r="B74" s="46">
         <f>SUM(N74:Q74)</f>
@@ -7558,7 +7623,7 @@
     </row>
     <row r="75" ht="61.5" customHeight="1" s="29">
       <c r="A75" s="45" t="n">
-        <v>71</v>
+        <v>79</v>
       </c>
       <c r="B75" s="46">
         <f>SUM(N75:Q75)</f>
@@ -7650,7 +7715,7 @@
     </row>
     <row r="76" ht="61.5" customHeight="1" s="29">
       <c r="A76" s="45" t="n">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="B76" s="46">
         <f>SUM(N76:Q76)</f>
@@ -7744,70 +7809,756 @@
         </is>
       </c>
     </row>
-    <row r="78" ht="15" customHeight="1" s="29">
-      <c r="A78" s="47" t="inlineStr">
-        <is>
-          <t>Total des occasions</t>
-        </is>
-      </c>
-      <c r="B78" s="47">
-        <f>COUNTA(D5:D76)</f>
+    <row r="77" ht="62" customHeight="1" s="29">
+      <c r="A77" s="60" t="n">
+        <v>7</v>
+      </c>
+      <c r="B77" s="61">
+        <f>SUM(N77:Q77)</f>
         <v/>
       </c>
-    </row>
-    <row r="79" ht="15" customHeight="1" s="29">
-      <c r="A79" s="48" t="inlineStr">
-        <is>
-          <t>Priorité A</t>
-        </is>
-      </c>
-      <c r="B79" s="48">
-        <f>COUNTIF(C5:C76,"A")</f>
+      <c r="C77" s="61" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D77" s="62" t="inlineStr">
+        <is>
+          <t>Gourmet Sauvage</t>
+        </is>
+      </c>
+      <c r="E77" s="63" t="inlineStr">
+        <is>
+          <t>https://gourmetsauvage.ca/</t>
+        </is>
+      </c>
+      <c r="F77" s="64" t="inlineStr">
+        <is>
+          <t>Partenaire de filière, asclépiade comestible</t>
+        </is>
+      </c>
+      <c r="G77" s="64" t="inlineStr">
+        <is>
+          <t>Ajout du 3 août 2026</t>
+        </is>
+      </c>
+      <c r="H77" s="64" t="inlineStr">
+        <is>
+          <t>Entreprise des Laurentides, 30 ans de cueillette sauvage, fondée par Gérald Le Gal et reprise par Ariane Paré-Le Gal. Vend des gousses d'asclépiade marinées et donne des ateliers de cueillette.</t>
+        </is>
+      </c>
+      <c r="I77" s="64" t="inlineStr">
+        <is>
+          <t>Page pilier asclépiade + page mission</t>
+        </is>
+      </c>
+      <c r="J77" s="64" t="inlineStr">
+        <is>
+          <t>La complémentarité la plus nette de tout l'audit : ils utilisent la pousse, le bouton et la jeune gousse, Lasclay utilise la soie du follicule mûr. Aucune concurrence, la même plante, deux saisons différentes. Proposer un contenu croisé sur le cycle complet de la plante.</t>
+        </is>
+      </c>
+      <c r="K77" s="64" t="inlineStr">
+        <is>
+          <t>À trouver</t>
+        </is>
+      </c>
+      <c r="L77" s="64" t="inlineStr">
+        <is>
+          <t>À trouver (formulaire de contact)</t>
+        </is>
+      </c>
+      <c r="M77" s="64" t="inlineStr">
+        <is>
+          <t>gourmetsauvage.ca/en/contact/ | Saint-Faustin-Lac-Carré, Laurentides</t>
+        </is>
+      </c>
+      <c r="N77" s="60" t="n">
+        <v>29</v>
+      </c>
+      <c r="O77" s="60" t="n">
+        <v>18</v>
+      </c>
+      <c r="P77" s="60" t="n">
+        <v>20</v>
+      </c>
+      <c r="Q77" s="60" t="n">
+        <v>15</v>
+      </c>
+      <c r="R77" s="64" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+      <c r="S77" s="64" t="inlineStr">
+        <is>
+          <t>Angle éditorial fort : une seule plante, deux usages, zéro concurrence.</t>
+        </is>
+      </c>
+      <c r="T77" s="62" t="inlineStr">
+        <is>
+          <t>NON, aucune mention ni lien (vérifié le 3 août 2026)</t>
+        </is>
+      </c>
+      <c r="U77" s="64" t="inlineStr">
+        <is>
+          <t>Occasion à qualifier puis à contacter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="62" customHeight="1" s="29">
+      <c r="A78" s="60" t="n">
+        <v>23</v>
+      </c>
+      <c r="B78" s="61">
+        <f>SUM(N78:Q78)</f>
         <v/>
       </c>
-    </row>
-    <row r="80" ht="15" customHeight="1" s="29">
-      <c r="A80" s="48" t="inlineStr">
-        <is>
-          <t>Priorité B</t>
-        </is>
-      </c>
-      <c r="B80" s="48">
-        <f>COUNTIF(C5:C76,"B")</f>
+      <c r="C78" s="61" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D78" s="62" t="inlineStr">
+        <is>
+          <t>Symbiose Herboristerie</t>
+        </is>
+      </c>
+      <c r="E78" s="63" t="inlineStr">
+        <is>
+          <t>https://www.symbioseherboristerie.com/blogue/lasclepiade-en-cuisine/</t>
+        </is>
+      </c>
+      <c r="F78" s="64" t="inlineStr">
+        <is>
+          <t>Mention existante, blogue</t>
+        </is>
+      </c>
+      <c r="G78" s="64" t="inlineStr">
+        <is>
+          <t>Ajout du 3 août 2026</t>
+        </is>
+      </c>
+      <c r="H78" s="64" t="inlineStr">
+        <is>
+          <t>Article « L'asclépiade en cuisine ».</t>
+        </is>
+      </c>
+      <c r="I78" s="64" t="inlineStr">
+        <is>
+          <t>Page pilier asclépiade</t>
+        </is>
+      </c>
+      <c r="J78" s="64" t="inlineStr">
+        <is>
+          <t>Rien à demander, le lien est déjà là. Remercier et entretenir la relation.</t>
+        </is>
+      </c>
+      <c r="K78" s="64" t="inlineStr">
+        <is>
+          <t>À trouver</t>
+        </is>
+      </c>
+      <c r="L78" s="64" t="inlineStr">
+        <is>
+          <t>À trouver (page de contact)</t>
+        </is>
+      </c>
+      <c r="M78" s="64" t="inlineStr">
+        <is>
+          <t>symbioseherboristerie.com/contact/</t>
+        </is>
+      </c>
+      <c r="N78" s="60" t="n">
+        <v>28</v>
+      </c>
+      <c r="O78" s="60" t="n">
+        <v>12</v>
+      </c>
+      <c r="P78" s="60" t="n">
+        <v>25</v>
+      </c>
+      <c r="Q78" s="60" t="n">
+        <v>13</v>
+      </c>
+      <c r="R78" s="64" t="inlineStr">
+        <is>
+          <t>Lien obtenu</t>
+        </is>
+      </c>
+      <c r="S78" s="64" t="inlineStr">
+        <is>
+          <t>Découvert hors de l'audit initial. Te liait déjà sans que ce soit su.</t>
+        </is>
+      </c>
+      <c r="T78" s="65" t="inlineStr">
+        <is>
+          <t>OUI, lien en place (vérifié le 3 août 2026)</t>
+        </is>
+      </c>
+      <c r="U78" s="64" t="inlineStr">
+        <is>
+          <t>Rien à demander, le lien est déjà en place.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="62" customHeight="1" s="29">
+      <c r="A79" s="66" t="n">
+        <v>50</v>
+      </c>
+      <c r="B79" s="67">
+        <f>SUM(N79:Q79)</f>
         <v/>
       </c>
-    </row>
-    <row r="81" ht="15" customHeight="1" s="29">
-      <c r="A81" s="48" t="inlineStr">
-        <is>
-          <t>Priorité C</t>
-        </is>
-      </c>
-      <c r="B81" s="48">
-        <f>COUNTIF(C5:C76,"C")</f>
+      <c r="C79" s="67" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D79" s="62" t="inlineStr">
+        <is>
+          <t>Herbasimple</t>
+        </is>
+      </c>
+      <c r="E79" s="63" t="inlineStr">
+        <is>
+          <t>https://herbasimple.com/blog/asclepiade-commune-toxique-ou-comestible/</t>
+        </is>
+      </c>
+      <c r="F79" s="64" t="inlineStr">
+        <is>
+          <t>Page ressource, asclépiade</t>
+        </is>
+      </c>
+      <c r="G79" s="64" t="inlineStr">
+        <is>
+          <t>Ajout du 3 août 2026</t>
+        </is>
+      </c>
+      <c r="H79" s="64" t="inlineStr">
+        <is>
+          <t>Article « Asclépiade commune : toxique ou comestible ? ».</t>
+        </is>
+      </c>
+      <c r="I79" s="64" t="inlineStr">
+        <is>
+          <t>Page pilier asclépiade</t>
+        </is>
+      </c>
+      <c r="J79" s="64" t="inlineStr">
+        <is>
+          <t>Sujet voisin, public curieux de la plante. Proposer la page pilier en complément botanique.</t>
+        </is>
+      </c>
+      <c r="K79" s="64" t="inlineStr">
+        <is>
+          <t>À trouver</t>
+        </is>
+      </c>
+      <c r="L79" s="64" t="inlineStr">
+        <is>
+          <t>À trouver (page de contact)</t>
+        </is>
+      </c>
+      <c r="M79" s="64" t="inlineStr">
+        <is>
+          <t>herbasimple.com</t>
+        </is>
+      </c>
+      <c r="N79" s="66" t="n">
+        <v>26</v>
+      </c>
+      <c r="O79" s="66" t="n">
+        <v>12</v>
+      </c>
+      <c r="P79" s="66" t="n">
+        <v>20</v>
+      </c>
+      <c r="Q79" s="66" t="n">
+        <v>11</v>
+      </c>
+      <c r="R79" s="64" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+      <c r="S79" s="64" t="inlineStr"/>
+      <c r="T79" s="62" t="inlineStr">
+        <is>
+          <t>NON, aucune mention ni lien (vérifié le 3 août 2026)</t>
+        </is>
+      </c>
+      <c r="U79" s="64" t="inlineStr">
+        <is>
+          <t>Occasion à qualifier puis à contacter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="62" customHeight="1" s="29">
+      <c r="A80" s="66" t="n">
+        <v>53</v>
+      </c>
+      <c r="B80" s="67">
+        <f>SUM(N80:Q80)</f>
         <v/>
       </c>
-    </row>
-    <row r="82" ht="15" customHeight="1" s="29">
-      <c r="A82" s="48" t="inlineStr">
-        <is>
-          <t>Courriels confirmés</t>
-        </is>
-      </c>
-      <c r="B82" s="48">
-        <f>COUNTIF(L5:L76,"Confirmé*")</f>
+      <c r="C80" s="67" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D80" s="62" t="inlineStr">
+        <is>
+          <t>Banlieusardises</t>
+        </is>
+      </c>
+      <c r="E80" s="63" t="inlineStr">
+        <is>
+          <t>https://www.banlieusardises.com/gousses-dasclepiades-sautees-au-beurre/</t>
+        </is>
+      </c>
+      <c r="F80" s="64" t="inlineStr">
+        <is>
+          <t>Page ressource, recette</t>
+        </is>
+      </c>
+      <c r="G80" s="64" t="inlineStr">
+        <is>
+          <t>Ajout du 3 août 2026</t>
+        </is>
+      </c>
+      <c r="H80" s="64" t="inlineStr">
+        <is>
+          <t>Recette de gousses d'asclépiades sautées au beurre sur un blogue québécois de longue date.</t>
+        </is>
+      </c>
+      <c r="I80" s="64" t="inlineStr">
+        <is>
+          <t>Page pilier asclépiade</t>
+        </is>
+      </c>
+      <c r="J80" s="64" t="inlineStr">
+        <is>
+          <t>Blogue personnel établi, facile à joindre. Offrir la ressource botanique en complément de la recette.</t>
+        </is>
+      </c>
+      <c r="K80" s="64" t="inlineStr">
+        <is>
+          <t>À trouver</t>
+        </is>
+      </c>
+      <c r="L80" s="64" t="inlineStr">
+        <is>
+          <t>À trouver (page de contact)</t>
+        </is>
+      </c>
+      <c r="M80" s="64" t="inlineStr">
+        <is>
+          <t>banlieusardises.com</t>
+        </is>
+      </c>
+      <c r="N80" s="66" t="n">
+        <v>24</v>
+      </c>
+      <c r="O80" s="66" t="n">
+        <v>13</v>
+      </c>
+      <c r="P80" s="66" t="n">
+        <v>21</v>
+      </c>
+      <c r="Q80" s="66" t="n">
+        <v>10</v>
+      </c>
+      <c r="R80" s="64" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+      <c r="S80" s="64" t="inlineStr"/>
+      <c r="T80" s="62" t="inlineStr">
+        <is>
+          <t>NON, aucune mention ni lien (vérifié le 3 août 2026)</t>
+        </is>
+      </c>
+      <c r="U80" s="64" t="inlineStr">
+        <is>
+          <t>Occasion à qualifier puis à contacter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="62" customHeight="1" s="29">
+      <c r="A81" s="66" t="n">
+        <v>45</v>
+      </c>
+      <c r="B81" s="67">
+        <f>SUM(N81:Q81)</f>
         <v/>
       </c>
-    </row>
-    <row r="83" ht="15" customHeight="1" s="29">
-      <c r="A83" s="47" t="inlineStr">
-        <is>
-          <t>Liens obtenus</t>
-        </is>
-      </c>
-      <c r="B83" s="47">
-        <f>COUNTIF(R5:R76,"Lien obtenu")</f>
+      <c r="C81" s="67" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D81" s="62" t="inlineStr">
+        <is>
+          <t>La Presse (asclépiade comestible, 2014)</t>
+        </is>
+      </c>
+      <c r="E81" s="63" t="inlineStr">
+        <is>
+          <t>https://www.lapresse.ca/vivre/gourmand/cuisine/terroir/201407/31/01-4788196-decouvrir-lasclepiade-commune.php</t>
+        </is>
+      </c>
+      <c r="F81" s="64" t="inlineStr">
+        <is>
+          <t>Presse nationale, sujet asclépiade</t>
+        </is>
+      </c>
+      <c r="G81" s="64" t="inlineStr">
+        <is>
+          <t>Ajout du 3 août 2026</t>
+        </is>
+      </c>
+      <c r="H81" s="64" t="inlineStr">
+        <is>
+          <t>Article « Découvrir l'asclépiade commune » dans la section terroir.</t>
+        </is>
+      </c>
+      <c r="I81" s="64" t="inlineStr">
+        <is>
+          <t>Page pilier asclépiade</t>
+        </is>
+      </c>
+      <c r="J81" s="64" t="inlineStr">
+        <is>
+          <t>Article ancien. Se rendre disponible comme source pour une reprise du sujet.</t>
+        </is>
+      </c>
+      <c r="K81" s="64" t="inlineStr">
+        <is>
+          <t>À trouver</t>
+        </is>
+      </c>
+      <c r="L81" s="64" t="inlineStr">
+        <is>
+          <t>À trouver (contacter la ou le signataire)</t>
+        </is>
+      </c>
+      <c r="M81" s="64" t="inlineStr"/>
+      <c r="N81" s="66" t="n">
+        <v>24</v>
+      </c>
+      <c r="O81" s="66" t="n">
+        <v>25</v>
+      </c>
+      <c r="P81" s="66" t="n">
+        <v>9</v>
+      </c>
+      <c r="Q81" s="66" t="n">
+        <v>12</v>
+      </c>
+      <c r="R81" s="64" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+      <c r="S81" s="64" t="inlineStr">
+        <is>
+          <t>Angle alimentaire, pas textile. Public différent mais même plante.</t>
+        </is>
+      </c>
+      <c r="T81" s="62" t="inlineStr">
+        <is>
+          <t>NON, aucune mention ni lien (vérifié le 3 août 2026)</t>
+        </is>
+      </c>
+      <c r="U81" s="64" t="inlineStr">
+        <is>
+          <t>Occasion à qualifier puis à contacter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="62" customHeight="1" s="29">
+      <c r="A82" s="66" t="n">
+        <v>46</v>
+      </c>
+      <c r="B82" s="67">
+        <f>SUM(N82:Q82)</f>
         <v/>
+      </c>
+      <c r="C82" s="67" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D82" s="62" t="inlineStr">
+        <is>
+          <t>Lufa (blogue)</t>
+        </is>
+      </c>
+      <c r="E82" s="63" t="inlineStr">
+        <is>
+          <t>https://montreal.lufa.com/fr/blog/recettes/apprivoiser-les-aliments-sauvages-tresors-et-recettes-de-gourmet-sauvage</t>
+        </is>
+      </c>
+      <c r="F82" s="64" t="inlineStr">
+        <is>
+          <t>Blogue de marque, aliments sauvages</t>
+        </is>
+      </c>
+      <c r="G82" s="64" t="inlineStr">
+        <is>
+          <t>Ajout du 3 août 2026</t>
+        </is>
+      </c>
+      <c r="H82" s="64" t="inlineStr">
+        <is>
+          <t>Billet sur les aliments sauvages avec Gourmet Sauvage. Grande plateforme d'agriculture urbaine à Montréal.</t>
+        </is>
+      </c>
+      <c r="I82" s="64" t="inlineStr">
+        <is>
+          <t>Page pilier asclépiade + collection semences</t>
+        </is>
+      </c>
+      <c r="J82" s="64" t="inlineStr">
+        <is>
+          <t>Angle partenariat plutôt que lien : ils ont un programme de partenaires et des points de chute.</t>
+        </is>
+      </c>
+      <c r="K82" s="64" t="inlineStr">
+        <is>
+          <t>partenaires@lufa.com</t>
+        </is>
+      </c>
+      <c r="L82" s="64" t="inlineStr">
+        <is>
+          <t>Confirmé</t>
+        </is>
+      </c>
+      <c r="M82" s="64" t="inlineStr">
+        <is>
+          <t>pointsdechute@lufa.com</t>
+        </is>
+      </c>
+      <c r="N82" s="66" t="n">
+        <v>20</v>
+      </c>
+      <c r="O82" s="66" t="n">
+        <v>20</v>
+      </c>
+      <c r="P82" s="66" t="n">
+        <v>16</v>
+      </c>
+      <c r="Q82" s="66" t="n">
+        <v>14</v>
+      </c>
+      <c r="R82" s="64" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+      <c r="S82" s="64" t="inlineStr">
+        <is>
+          <t>Piste commerciale autant que piste de lien.</t>
+        </is>
+      </c>
+      <c r="T82" s="62" t="inlineStr">
+        <is>
+          <t>NON, aucune mention ni lien (vérifié le 3 août 2026)</t>
+        </is>
+      </c>
+      <c r="U82" s="64" t="inlineStr">
+        <is>
+          <t>Occasion à qualifier puis à contacter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="62" customHeight="1" s="29">
+      <c r="A83" s="68" t="n">
+        <v>73</v>
+      </c>
+      <c r="B83" s="69">
+        <f>SUM(N83:Q83)</f>
+        <v/>
+      </c>
+      <c r="C83" s="69" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D83" s="62" t="inlineStr">
+        <is>
+          <t>Journal Le Tour</t>
+        </is>
+      </c>
+      <c r="E83" s="63" t="inlineStr">
+        <is>
+          <t>https://journalletour.com/plantes-sauvages-comestibles/</t>
+        </is>
+      </c>
+      <c r="F83" s="64" t="inlineStr">
+        <is>
+          <t>Média local, plantes sauvages</t>
+        </is>
+      </c>
+      <c r="G83" s="64" t="inlineStr">
+        <is>
+          <t>Ajout du 3 août 2026</t>
+        </is>
+      </c>
+      <c r="H83" s="64" t="inlineStr">
+        <is>
+          <t>Article sur les plantes sauvages comestibles du printemps.</t>
+        </is>
+      </c>
+      <c r="I83" s="64" t="inlineStr">
+        <is>
+          <t>Page pilier asclépiade</t>
+        </is>
+      </c>
+      <c r="J83" s="64" t="inlineStr">
+        <is>
+          <t>Petit média accessible. Offrir un contenu sur l'asclépiade au-delà de l'assiette.</t>
+        </is>
+      </c>
+      <c r="K83" s="64" t="inlineStr">
+        <is>
+          <t>annieaire@gmail.com</t>
+        </is>
+      </c>
+      <c r="L83" s="64" t="inlineStr">
+        <is>
+          <t>Confirmé (trouvé sur la page)</t>
+        </is>
+      </c>
+      <c r="M83" s="64" t="inlineStr">
+        <is>
+          <t>journalletour.com</t>
+        </is>
+      </c>
+      <c r="N83" s="68" t="n">
+        <v>20</v>
+      </c>
+      <c r="O83" s="68" t="n">
+        <v>9</v>
+      </c>
+      <c r="P83" s="68" t="n">
+        <v>22</v>
+      </c>
+      <c r="Q83" s="68" t="n">
+        <v>8</v>
+      </c>
+      <c r="R83" s="64" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+      <c r="S83" s="64" t="inlineStr"/>
+      <c r="T83" s="62" t="inlineStr">
+        <is>
+          <t>NON, aucune mention ni lien (vérifié le 3 août 2026)</t>
+        </is>
+      </c>
+      <c r="U83" s="64" t="inlineStr">
+        <is>
+          <t>Occasion à qualifier puis à contacter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="62" customHeight="1" s="29">
+      <c r="A84" s="66" t="n">
+        <v>30</v>
+      </c>
+      <c r="B84" s="67">
+        <f>SUM(N84:Q84)</f>
+        <v/>
+      </c>
+      <c r="C84" s="67" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D84" s="62" t="inlineStr">
+        <is>
+          <t>Unpointcinq</t>
+        </is>
+      </c>
+      <c r="E84" s="63" t="inlineStr">
+        <is>
+          <t>https://unpointcinq.ca/agir/plantes-sauvages-comestibles-quebec/</t>
+        </is>
+      </c>
+      <c r="F84" s="64" t="inlineStr">
+        <is>
+          <t>Média climat, plantes sauvages</t>
+        </is>
+      </c>
+      <c r="G84" s="64" t="inlineStr">
+        <is>
+          <t>Ajout du 3 août 2026</t>
+        </is>
+      </c>
+      <c r="H84" s="64" t="inlineStr">
+        <is>
+          <t>Article « Savez-vous manger les plantes, à la mode de chez nous ? ». Média québécois consacré à l'action climatique.</t>
+        </is>
+      </c>
+      <c r="I84" s="64" t="inlineStr">
+        <is>
+          <t>Page mission + page pilier asclépiade</t>
+        </is>
+      </c>
+      <c r="J84" s="64" t="inlineStr">
+        <is>
+          <t>Média dont la ligne éditoriale colle exactement à la mission de Lasclay. Proposer un sujet sur la culture de l'asclépiade comme levier d'habitat.</t>
+        </is>
+      </c>
+      <c r="K84" s="64" t="inlineStr">
+        <is>
+          <t>À trouver</t>
+        </is>
+      </c>
+      <c r="L84" s="64" t="inlineStr">
+        <is>
+          <t>À trouver (rédaction)</t>
+        </is>
+      </c>
+      <c r="M84" s="64" t="inlineStr">
+        <is>
+          <t>unpointcinq.ca</t>
+        </is>
+      </c>
+      <c r="N84" s="66" t="n">
+        <v>26</v>
+      </c>
+      <c r="O84" s="66" t="n">
+        <v>19</v>
+      </c>
+      <c r="P84" s="66" t="n">
+        <v>16</v>
+      </c>
+      <c r="Q84" s="66" t="n">
+        <v>14</v>
+      </c>
+      <c r="R84" s="64" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+      <c r="S84" s="64" t="inlineStr">
+        <is>
+          <t>Un des meilleurs alignements éditoriaux du lot.</t>
+        </is>
+      </c>
+      <c r="T84" s="62" t="inlineStr">
+        <is>
+          <t>NON, aucune mention ni lien (vérifié le 3 août 2026)</t>
+        </is>
+      </c>
+      <c r="U84" s="64" t="inlineStr">
+        <is>
+          <t>Occasion à qualifier puis à contacter.</t>
+        </is>
       </c>
     </row>
     <row r="85" ht="15" customHeight="1" s="29">
@@ -7866,7 +8617,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:U76"/>
+  <autoFilter ref="A4:U84"/>
   <mergeCells count="2">
     <mergeCell ref="A2:S2"/>
     <mergeCell ref="A1:S1"/>
@@ -7953,6 +8704,14 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E74" display="https://www.madetomeasuremag.com/vegeto-launches-sustainable-heavy-duty-insulation-material-made-of-milkweed" r:id="rId70"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E75" display="https://lemarcheauxtresors.company.site/" r:id="rId71"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E76" display="https://www.lhebdodustmaurice.com/actualites/nouveau-partenaire-developpement-de-lasclepiade/" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E77" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E78" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E79" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E80" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E81" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E82" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E83" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E84" r:id="rId80"/>
   </hyperlinks>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>